<commit_message>
chore: monthly review 2026-09-25 23:01Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/monthly_review.xlsx
+++ b/public/monthly_review.xlsx
@@ -1270,11 +1270,11 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D17" s="34" t="n">
-        <v>-2.61</v>
+        <v>-4.49</v>
       </c>
     </row>
     <row r="18">
@@ -13282,7 +13282,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DC07DC6C-31A3-40B8-B518-5041140083C4}</x14:id>
+          <x14:id>{93E268D4-C5F1-4C4E-B644-9BF36B5A1229}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -13296,7 +13296,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{38AE9222-224D-45F8-A48E-9BE78F9FB682}</x14:id>
+          <x14:id>{BE1E5884-4C31-4BF7-91F9-6BDC80E4E4E6}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -13310,7 +13310,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6BDB3E11-5A87-4205-A792-57BE64617593}</x14:id>
+          <x14:id>{B551D18A-631D-4A32-8634-797F2CACA18B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -13324,7 +13324,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0469EFAF-31B9-40FD-AD0A-6B1A0D046D6C}</x14:id>
+          <x14:id>{EDF90DEE-0094-4DCD-8507-2EE5F6B352A8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -13334,7 +13334,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DC07DC6C-31A3-40B8-B518-5041140083C4}">
+          <x14:cfRule type="dataBar" id="{93E268D4-C5F1-4C4E-B644-9BF36B5A1229}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -13347,7 +13347,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{38AE9222-224D-45F8-A48E-9BE78F9FB682}">
+          <x14:cfRule type="dataBar" id="{BE1E5884-4C31-4BF7-91F9-6BDC80E4E4E6}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -13360,7 +13360,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6BDB3E11-5A87-4205-A792-57BE64617593}">
+          <x14:cfRule type="dataBar" id="{B551D18A-631D-4A32-8634-797F2CACA18B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -13373,7 +13373,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0469EFAF-31B9-40FD-AD0A-6B1A0D046D6C}">
+          <x14:cfRule type="dataBar" id="{EDF90DEE-0094-4DCD-8507-2EE5F6B352A8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: monthly review 2026-10-16 23:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/monthly_review.xlsx
+++ b/public/monthly_review.xlsx
@@ -1017,7 +1017,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 09/30 → 10/15, %</t>
+          <t>미국 종가 기준 09/30 → 10/16, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1087,19 +1087,19 @@
         <v>17552</v>
       </c>
       <c r="E8" s="28" t="n">
-        <v>1.21</v>
+        <v>0.1</v>
       </c>
       <c r="F8" s="28" t="n">
-        <v>2.5</v>
+        <v>2.15</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>-0.55</v>
+        <v>-2.68</v>
       </c>
       <c r="H8" s="28" t="n">
-        <v>0.73</v>
+        <v>22.34</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>-8.289999999999999</v>
+        <v>-11.81</v>
       </c>
     </row>
     <row r="9">
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>8.23</v>
+        <v>10.96</v>
       </c>
     </row>
     <row r="13">
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>5.21</v>
+        <v>4.92</v>
       </c>
     </row>
     <row r="14">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>임의소비재</t>
+          <t>소재</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>4.2</v>
+        <v>4.56</v>
       </c>
     </row>
     <row r="15">
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-8.24</v>
+        <v>-11.36</v>
       </c>
     </row>
     <row r="16">
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-5.01</v>
+        <v>-8.470000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-3.35</v>
+        <v>-6.27</v>
       </c>
     </row>
     <row r="18">
@@ -12533,7 +12533,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6465E6DC-CF2B-4C89-947F-3C7E1FAE49B7}</x14:id>
+          <x14:id>{FECEE320-D8CE-4176-B9EA-F2F666A6397E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12547,7 +12547,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F9C1BF1-E0A5-4A2F-8A0E-4A5314356E37}</x14:id>
+          <x14:id>{55ED9D88-4BB3-4B27-8CDC-7EE36578434B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12561,7 +12561,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FF5AB180-D82C-4CA9-BA4D-360D9676F114}</x14:id>
+          <x14:id>{66E522BF-8341-4D54-A5B0-2C111935C0D8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12575,7 +12575,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A01ECB40-8140-4E1E-807F-858515B874C9}</x14:id>
+          <x14:id>{40744A85-887D-41DF-8BE7-FE8C45BE0F7B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12585,7 +12585,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6465E6DC-CF2B-4C89-947F-3C7E1FAE49B7}">
+          <x14:cfRule type="dataBar" id="{FECEE320-D8CE-4176-B9EA-F2F666A6397E}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12598,7 +12598,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F9C1BF1-E0A5-4A2F-8A0E-4A5314356E37}">
+          <x14:cfRule type="dataBar" id="{55ED9D88-4BB3-4B27-8CDC-7EE36578434B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12611,7 +12611,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FF5AB180-D82C-4CA9-BA4D-360D9676F114}">
+          <x14:cfRule type="dataBar" id="{66E522BF-8341-4D54-A5B0-2C111935C0D8}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12624,7 +12624,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A01ECB40-8140-4E1E-807F-858515B874C9}">
+          <x14:cfRule type="dataBar" id="{40744A85-887D-41DF-8BE7-FE8C45BE0F7B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>

<commit_message>
chore: monthly review 2026-10-23 23:01Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/monthly_review.xlsx
+++ b/public/monthly_review.xlsx
@@ -1020,7 +1020,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 09/30 → 10/22, %</t>
+          <t>미국 종가 기준 09/30 → 10/23, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1089,20 +1089,20 @@
       <c r="D8" s="28" t="n">
         <v>16699</v>
       </c>
-      <c r="E8" s="28" t="n">
-        <v>0.16</v>
+      <c r="E8" s="29" t="n">
+        <v>-0.36</v>
       </c>
       <c r="F8" s="28" t="n">
-        <v>3.85</v>
+        <v>2.57</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>-3.17</v>
+        <v>-3.37</v>
       </c>
       <c r="H8" s="28" t="n">
-        <v>16.46</v>
+        <v>19.03</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>-15.02</v>
+        <v>-14.64</v>
       </c>
     </row>
     <row r="9">
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>9.869999999999999</v>
+        <v>12.73</v>
       </c>
     </row>
     <row r="13">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>7.65</v>
+        <v>6.45</v>
       </c>
     </row>
     <row r="14">
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>6.14</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="15">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-14.06</v>
+        <v>-13.43</v>
       </c>
     </row>
     <row r="16">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-6.85</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="17">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-3.83</v>
+        <v>-5.16</v>
       </c>
     </row>
     <row r="18">
@@ -12844,7 +12844,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{EE7B8045-EC19-4BB5-A7D8-263B480F321A}</x14:id>
+          <x14:id>{6D10690F-C0E0-401B-89F2-5DF5250FF68A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12858,7 +12858,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D0453A34-5CBF-4CF6-BC3D-690832AF9BA8}</x14:id>
+          <x14:id>{DA02D0B1-F057-4961-AC2E-F305DD077A83}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12872,7 +12872,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E295493-1FE4-4B04-9291-6DF389B0BD12}</x14:id>
+          <x14:id>{7EAF0C9F-D299-420A-A99E-2CA80C11B20C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12886,7 +12886,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{01F5D576-07EB-4504-9791-8DF2EA397790}</x14:id>
+          <x14:id>{8CBE2EA4-B133-4411-B0D1-241C3F04C332}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12896,7 +12896,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{EE7B8045-EC19-4BB5-A7D8-263B480F321A}">
+          <x14:cfRule type="dataBar" id="{6D10690F-C0E0-401B-89F2-5DF5250FF68A}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12909,7 +12909,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D0453A34-5CBF-4CF6-BC3D-690832AF9BA8}">
+          <x14:cfRule type="dataBar" id="{DA02D0B1-F057-4961-AC2E-F305DD077A83}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12922,7 +12922,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E295493-1FE4-4B04-9291-6DF389B0BD12}">
+          <x14:cfRule type="dataBar" id="{7EAF0C9F-D299-420A-A99E-2CA80C11B20C}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -12935,7 +12935,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{01F5D576-07EB-4504-9791-8DF2EA397790}">
+          <x14:cfRule type="dataBar" id="{8CBE2EA4-B133-4411-B0D1-241C3F04C332}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>